<commit_message>
publish: workflow_dispatch ui-qol (442cbbb)
</commit_message>
<xml_diff>
--- a/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 442cbbb (built 2026-10-15 05:07 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 442cbbb (built 2026-10-15 05:08 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:07 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push ui-qol (352cfc1)
</commit_message>
<xml_diff>
--- a/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 442cbbb (built 2026-10-15 05:08 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 352cfc1 (built 2026-10-15 05:34 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 442cbbb · built 2026-10-15 05:08 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push ui-qol (596e550)
</commit_message>
<xml_diff>
--- a/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 352cfc1 (built 2026-10-15 05:34 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 596e550 (built 2026-10-15 06:02 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 352cfc1 · built 2026-10-15 05:34 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push ui-qol (79288c9)
</commit_message>
<xml_diff>
--- a/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 596e550 (built 2026-10-15 06:02 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 79288c9 (built 2026-10-15 06:24 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 596e550 · built 2026-10-15 06:02 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push ui-qol (4e28dd2)
</commit_message>
<xml_diff>
--- a/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 79288c9 (built 2026-10-15 06:24 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 4e28dd2 (built 2026-10-15 06:27 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 79288c9 · built 2026-10-15 06:24 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push ui-qol (0dcc109)
</commit_message>
<xml_diff>
--- a/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 4e28dd2 (built 2026-10-15 06:27 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 0dcc109 (built 2026-10-15 06:44 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 4e28dd2 · built 2026-10-15 06:27 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push ui-qol (f104f35)
</commit_message>
<xml_diff>
--- a/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch ui-qol · commit 0dcc109 (built 2026-10-15 06:44 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch ui-qol · commit f104f35 (built 2026-10-15 06:47 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7374,7 +7374,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12353,7 +12353,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14484,7 +14484,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27253,7 +27253,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28557,7 +28557,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29147,7 +29147,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32449,7 +32449,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33629,7 +33629,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35122,7 +35122,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37288,7 +37288,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42559,7 +42559,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46767,7 +46767,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit 0dcc109 · built 2026-10-15 06:44 UTC</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push ui-qol (a106d5d)
</commit_message>
<xml_diff>
--- a/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/ui-qol/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1776,7 +1776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:B131"/>
+  <dimension ref="B1:B129"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="124" min="1" max="1"/>
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch ui-qol · commit f104f35 (built 2026-10-15 06:47 UTC). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch ui-qol · commit a106d5d (built 2026-10-15 14:57 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2245,21 +2245,14 @@
     </row>
     <row r="129" ht="14.25" customHeight="1" s="125">
       <c r="B129" s="129" t="n"/>
-    </row>
-    <row r="131">
-      <c r="B131" s="129" t="inlineStr">
-        <is>
-          <t>License: Healthcare Interoperability Readiness Matrix for EMR Systems, Department of Health – Western Visayas Center for Health Development, licensed under CC BY 4.0 (https://creativecommons.org/licenses/by/4.0/).</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -7374,8 +7367,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -12353,8 +12346,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -14484,8 +14477,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -27253,8 +27246,8 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -28557,8 +28550,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -29147,8 +29140,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -32449,8 +32442,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -33629,8 +33622,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -35122,8 +35115,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -37288,8 +37281,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -42559,8 +42552,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -46767,8 +46760,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit f104f35 · built 2026-10-15 06:47 UTC</oddHeader>
-    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N&amp;R&amp;7 © DOH WV CHD · CC BY 4.0</oddFooter>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ui-qol · commit a106d5d · built 2026-10-15 14:57 PHT</oddHeader>
+    <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>